<commit_message>
Add dip weights to weight_data
</commit_message>
<xml_diff>
--- a/data/branch_weight_data_v0-1.xlsx
+++ b/data/branch_weight_data_v0-1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\McGrath\occ-coseismic\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4062F42-F262-46A4-BE72-FA3B65985B94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57EF525B-C3E7-4D1D-A918-5858FCE1E18F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-29550" yWindow="2115" windowWidth="28800" windowHeight="15345" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-105" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="all sheets" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,9 @@
     <sheet name="py_weights_4_0" sheetId="7" r:id="rId8"/>
     <sheet name="Sheet1" sheetId="6" r:id="rId9"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">crustal_weights_4_2!$L$1:$L$37</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -41,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="921" uniqueCount="311">
   <si>
     <t>N</t>
   </si>
@@ -971,6 +974,9 @@
   </si>
   <si>
     <t>dip_model</t>
+  </si>
+  <si>
+    <t>dip_weight</t>
   </si>
 </sst>
 </file>
@@ -4388,7 +4394,7 @@
         <v>0.505</v>
       </c>
       <c r="K2">
-        <f t="shared" ref="K2:K37" si="0">PRODUCT(G2:J2)</f>
+        <f>PRODUCT(G2:J2)</f>
         <v>3.1078962500000001E-2</v>
       </c>
       <c r="L2">
@@ -4447,7 +4453,7 @@
         <v>0.505</v>
       </c>
       <c r="K3">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="K2:K37" si="0">PRODUCT(G3:J3)</f>
         <v>1.279367E-2</v>
       </c>
       <c r="L3">
@@ -6275,7 +6281,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCFFA5B5-D9A2-4366-B369-676754E8E9F5}">
-  <dimension ref="A1:S10"/>
+  <dimension ref="A1:T10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.85546875" customWidth="1"/>
@@ -6284,13 +6290,13 @@
     <col min="5" max="5" width="11.42578125" customWidth="1"/>
     <col min="6" max="6" width="21.28515625" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="15" max="15" width="16.42578125" customWidth="1"/>
-    <col min="16" max="16" width="19.42578125" customWidth="1"/>
-    <col min="17" max="17" width="14.5703125" customWidth="1"/>
-    <col min="18" max="18" width="26.140625" customWidth="1"/>
+    <col min="16" max="16" width="16.42578125" customWidth="1"/>
+    <col min="17" max="17" width="19.42578125" customWidth="1"/>
+    <col min="18" max="18" width="14.5703125" customWidth="1"/>
+    <col min="19" max="19" width="26.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6325,31 +6331,34 @@
         <v>248</v>
       </c>
       <c r="L1" t="s">
+        <v>310</v>
+      </c>
+      <c r="M1" t="s">
         <v>249</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>254</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>256</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>259</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>264</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>4</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>188</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2.7</v>
       </c>
@@ -6384,28 +6393,31 @@
         <v>0.505</v>
       </c>
       <c r="L2">
-        <f t="shared" ref="L2" si="0">PRODUCT(H2:K2)</f>
-        <v>3.1078962500000001E-2</v>
+        <v>0.25</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <f>PRODUCT(H2:L2)</f>
+        <v>7.7697406250000003E-3</v>
       </c>
       <c r="N2">
-        <f>L2*M2</f>
-        <v>3.1078962500000001E-2</v>
+        <v>1</v>
       </c>
       <c r="O2">
-        <f>0.25*N2/SUM(N$4:N$10)</f>
-        <v>3.3577668643037413E-2</v>
-      </c>
-      <c r="P2" t="s">
+        <f>M2*N2</f>
+        <v>7.7697406250000003E-3</v>
+      </c>
+      <c r="P2">
+        <f>0.25*O2/SUM(O$2:O$10)</f>
+        <v>1.9850881036539765E-2</v>
+      </c>
+      <c r="Q2" t="s">
         <v>301</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2.7</v>
       </c>
@@ -6440,28 +6452,31 @@
         <v>0.505</v>
       </c>
       <c r="L3">
-        <f t="shared" ref="L3" si="1">PRODUCT(H3:K3)</f>
-        <v>3.1078962500000001E-2</v>
+        <v>0.25</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <f>PRODUCT(H3:L3)</f>
+        <v>7.7697406250000003E-3</v>
       </c>
       <c r="N3">
-        <f>L3*M3</f>
-        <v>3.1078962500000001E-2</v>
+        <v>1</v>
       </c>
       <c r="O3">
-        <f>0.25*N3/SUM(N$4:N$10)</f>
-        <v>3.3577668643037413E-2</v>
-      </c>
-      <c r="P3" t="s">
+        <f>M3*N3</f>
+        <v>7.7697406250000003E-3</v>
+      </c>
+      <c r="P3">
+        <f t="shared" ref="P3:P10" si="0">0.25*O3/SUM(O$2:O$10)</f>
+        <v>1.9850881036539765E-2</v>
+      </c>
+      <c r="Q3" t="s">
         <v>300</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2.7</v>
       </c>
@@ -6496,28 +6511,31 @@
         <v>0.505</v>
       </c>
       <c r="L4">
-        <f t="shared" ref="L4:L10" si="2">PRODUCT(H4:K4)</f>
-        <v>3.1078962500000001E-2</v>
+        <v>0.5</v>
       </c>
       <c r="M4">
-        <v>1</v>
+        <f>PRODUCT(H4:L4)</f>
+        <v>1.5539481250000001E-2</v>
       </c>
       <c r="N4">
-        <f>L4*M4</f>
-        <v>3.1078962500000001E-2</v>
+        <v>1</v>
       </c>
       <c r="O4">
-        <f>0.25*N4/SUM(N$4:N$10)</f>
-        <v>3.3577668643037413E-2</v>
-      </c>
-      <c r="P4" t="s">
+        <f>M4*N4</f>
+        <v>1.5539481250000001E-2</v>
+      </c>
+      <c r="P4">
+        <f t="shared" si="0"/>
+        <v>3.970176207307953E-2</v>
+      </c>
+      <c r="Q4" t="s">
         <v>302</v>
       </c>
-      <c r="R4" t="s">
+      <c r="S4" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3.4</v>
       </c>
@@ -6552,28 +6570,31 @@
         <v>0.505</v>
       </c>
       <c r="L5">
-        <f t="shared" ref="L5" si="3">PRODUCT(H5:K5)</f>
-        <v>6.9700100000000001E-2</v>
+        <v>0.25</v>
       </c>
       <c r="M5">
+        <f>PRODUCT(H5:L5)</f>
+        <v>1.7425025E-2</v>
+      </c>
+      <c r="N5">
         <v>0.748107262752845</v>
       </c>
-      <c r="N5">
-        <f t="shared" ref="N5" si="4">L5*M5</f>
-        <v>5.2143151024599571E-2</v>
-      </c>
       <c r="O5">
-        <f>0.25*N5/SUM(N$4:N$10)</f>
-        <v>5.6335389159398779E-2</v>
-      </c>
-      <c r="P5" t="s">
+        <f t="shared" ref="O5" si="1">M5*N5</f>
+        <v>1.3035787756149893E-2</v>
+      </c>
+      <c r="P5">
+        <f t="shared" si="0"/>
+        <v>3.3305085002745913E-2</v>
+      </c>
+      <c r="Q5" t="s">
         <v>303</v>
       </c>
-      <c r="R5" t="s">
+      <c r="S5" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>3.4</v>
       </c>
@@ -6608,28 +6629,31 @@
         <v>0.505</v>
       </c>
       <c r="L6">
-        <f t="shared" ref="L6" si="5">PRODUCT(H6:K6)</f>
-        <v>6.9700100000000001E-2</v>
+        <v>0.25</v>
       </c>
       <c r="M6">
+        <f>PRODUCT(H6:L6)</f>
+        <v>1.7425025E-2</v>
+      </c>
+      <c r="N6">
         <v>0.748107262752845</v>
       </c>
-      <c r="N6">
-        <f t="shared" ref="N6" si="6">L6*M6</f>
-        <v>5.2143151024599571E-2</v>
-      </c>
       <c r="O6">
-        <f>0.25*N6/SUM(N$4:N$10)</f>
-        <v>5.6335389159398779E-2</v>
-      </c>
-      <c r="P6" t="s">
+        <f t="shared" ref="O6" si="2">M6*N6</f>
+        <v>1.3035787756149893E-2</v>
+      </c>
+      <c r="P6">
+        <f t="shared" si="0"/>
+        <v>3.3305085002745913E-2</v>
+      </c>
+      <c r="Q6" t="s">
         <v>304</v>
       </c>
-      <c r="R6" t="s">
+      <c r="S6" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>3.4</v>
       </c>
@@ -6664,28 +6688,31 @@
         <v>0.505</v>
       </c>
       <c r="L7">
-        <f t="shared" si="2"/>
-        <v>6.9700100000000001E-2</v>
+        <v>0.5</v>
       </c>
       <c r="M7">
+        <f>PRODUCT(H7:L7)</f>
+        <v>3.485005E-2</v>
+      </c>
+      <c r="N7">
         <v>0.748107262752845</v>
       </c>
-      <c r="N7">
-        <f t="shared" ref="N7:N10" si="7">L7*M7</f>
-        <v>5.2143151024599571E-2</v>
-      </c>
       <c r="O7">
-        <f>0.25*N7/SUM(N$4:N$10)</f>
-        <v>5.6335389159398779E-2</v>
-      </c>
-      <c r="P7" t="s">
+        <f t="shared" ref="O7:O10" si="3">M7*N7</f>
+        <v>2.6071575512299786E-2</v>
+      </c>
+      <c r="P7">
+        <f t="shared" si="0"/>
+        <v>6.6610170005491826E-2</v>
+      </c>
+      <c r="Q7" t="s">
         <v>305</v>
       </c>
-      <c r="R7" t="s">
+      <c r="S7" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>4.5999999999999996</v>
       </c>
@@ -6720,28 +6747,31 @@
         <v>0.505</v>
       </c>
       <c r="L8">
-        <f t="shared" ref="L8" si="8">PRODUCT(H8:K8)</f>
-        <v>2.9258437500000001E-2</v>
+        <v>0.25</v>
       </c>
       <c r="M8">
+        <f>PRODUCT(H8:L8)</f>
+        <v>7.3146093750000004E-3</v>
+      </c>
+      <c r="N8">
         <v>0.5</v>
       </c>
-      <c r="N8">
-        <f t="shared" ref="N8" si="9">L8*M8</f>
-        <v>1.4629218750000001E-2</v>
-      </c>
       <c r="O8">
-        <f>0.25*N8/SUM(N$4:N$10)</f>
-        <v>1.5805387959588742E-2</v>
-      </c>
-      <c r="P8" t="s">
+        <f t="shared" ref="O8" si="4">M8*N8</f>
+        <v>3.6573046875000002E-3</v>
+      </c>
+      <c r="P8">
+        <f t="shared" si="0"/>
+        <v>9.3440339607143239E-3</v>
+      </c>
+      <c r="Q8" t="s">
         <v>306</v>
       </c>
-      <c r="R8" t="s">
+      <c r="S8" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>4.5999999999999996</v>
       </c>
@@ -6776,28 +6806,31 @@
         <v>0.505</v>
       </c>
       <c r="L9">
-        <f t="shared" ref="L9" si="10">PRODUCT(H9:K9)</f>
-        <v>2.9258437500000001E-2</v>
+        <v>0.25</v>
       </c>
       <c r="M9">
+        <f>PRODUCT(H9:L9)</f>
+        <v>7.3146093750000004E-3</v>
+      </c>
+      <c r="N9">
         <v>0.5</v>
       </c>
-      <c r="N9">
-        <f t="shared" ref="N9" si="11">L9*M9</f>
-        <v>1.4629218750000001E-2</v>
-      </c>
       <c r="O9">
-        <f>0.25*N9/SUM(N$4:N$10)</f>
-        <v>1.5805387959588742E-2</v>
-      </c>
-      <c r="P9" t="s">
+        <f t="shared" ref="O9" si="5">M9*N9</f>
+        <v>3.6573046875000002E-3</v>
+      </c>
+      <c r="P9">
+        <f t="shared" si="0"/>
+        <v>9.3440339607143239E-3</v>
+      </c>
+      <c r="Q9" t="s">
         <v>307</v>
       </c>
-      <c r="R9" t="s">
+      <c r="S9" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>4.5999999999999996</v>
       </c>
@@ -6832,24 +6865,27 @@
         <v>0.505</v>
       </c>
       <c r="L10">
-        <f t="shared" si="2"/>
-        <v>2.9258437500000001E-2</v>
+        <v>0.5</v>
       </c>
       <c r="M10">
+        <f>PRODUCT(H10:L10)</f>
+        <v>1.4629218750000001E-2</v>
+      </c>
+      <c r="N10">
         <v>0.5</v>
       </c>
-      <c r="N10">
-        <f t="shared" si="7"/>
-        <v>1.4629218750000001E-2</v>
-      </c>
       <c r="O10">
-        <f>0.25*N10/SUM(N$4:N$10)</f>
-        <v>1.5805387959588742E-2</v>
-      </c>
-      <c r="P10" t="s">
+        <f t="shared" si="3"/>
+        <v>7.3146093750000004E-3</v>
+      </c>
+      <c r="P10">
+        <f t="shared" si="0"/>
+        <v>1.8688067921428648E-2</v>
+      </c>
+      <c r="Q10" t="s">
         <v>308</v>
       </c>
-      <c r="R10" t="s">
+      <c r="S10" t="s">
         <v>299</v>
       </c>
     </row>

</xml_diff>